<commit_message>
Fix text layout in exported Excel workbooks
</commit_message>
<xml_diff>
--- a/examples/synthetic-results.xlsx
+++ b/examples/synthetic-results.xlsx
@@ -49,8 +49,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,338 +421,354 @@
   </sheetPr>
   <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="58" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="31" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>原始行号</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>导出用途</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>客户留言</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>联系方式</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>来源</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>意向等级</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>客户类型</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>线索阶段</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>客户回复</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>跟进动作</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>处理状态</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>判断依据</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>最终回复</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>回复状态</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>草稿-仅供复核</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>想采购100件，预算约2万元，多久能发货？</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>demo-contact-001</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>抖音</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>询价</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>新线索</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>您好，已了解您采购100件、预算约2万元。为了给您准备合适的报价，请问您关注的具体规格或型号是什么？</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>高优先级；确认规格或型号后，准备对应的报价信息。</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>成功</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
         <is>
           <t>包含询价或采购关键词</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="M2" s="1" t="inlineStr"/>
+      <c r="N2" s="1" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>草稿-仅供复核</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>我在杭州想做代理，怎么合作？</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>demo-contact-002</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>小红书</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>代理合作</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>新线索</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>您好，感谢您关注代理合作。了解到您所在地区是杭州，请问预计的合作规模如何？</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>高优先级；确认合作规模，准备代理政策和区域信息。</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>成功</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t>包含代理、合作或加盟关键词</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="M3" s="1" t="inlineStr"/>
+      <c r="N3" s="1" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>草稿-仅供复核</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>随便看看，先了解一下</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>demo-contact-003</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>网站</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>普通咨询</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>新线索</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>您好，感谢您的关注。您可以先了解产品信息，后续有具体需求时随时联系我们。</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="1" t="inlineStr">
         <is>
           <t>低优先级；记录兴趣，后续有新品或价格信息时再触达。</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="1" t="inlineStr">
         <is>
           <t>成功</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="1" t="inlineStr">
         <is>
           <t>表达了浏览或暂不决策意向</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="M4" s="1" t="inlineStr"/>
+      <c r="N4" s="1" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>草稿-仅供复核</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>订单号 A1008 的机器坏了，开机后无法使用。</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>demo-contact-004</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>公众号</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>售后</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="1" t="inlineStr">
         <is>
           <t>新线索</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>您好，已看到您的订单号 A1008。为了尽快帮您处理售后，请补充故障现象，方便我们核实。</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="1" t="inlineStr">
         <is>
           <t>优先跟进；核对订单并收集故障现象，交由售后确认。</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="1" t="inlineStr">
         <is>
           <t>成功</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" s="1" t="inlineStr">
         <is>
           <t>包含售后服务关键词</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="M5" s="1" t="inlineStr"/>
+      <c r="N5" s="1" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
@@ -768,206 +787,222 @@
   </sheetPr>
   <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="31" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>原始行号</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>导出用途</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>客户留言</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>联系方式</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>来源</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>意向等级</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>客户类型</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>线索阶段</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>客户回复</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>跟进动作</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>处理状态</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>判断依据</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>最终回复</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>回复状态</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>草稿-仅供复核</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>想采购100件，预算约2万元，多久能发货？</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>demo-contact-001</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>抖音</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>询价</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>新线索</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>您好，已了解您采购100件、预算约2万元。为了给您准备合适的报价，请问您关注的具体规格或型号是什么？</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>高优先级；确认规格或型号后，准备对应的报价信息。</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>成功</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
         <is>
           <t>包含询价或采购关键词</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="M2" s="1" t="inlineStr"/>
+      <c r="N2" s="1" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>草稿-仅供复核</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>我在杭州想做代理，怎么合作？</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>demo-contact-002</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>小红书</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>代理合作</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>新线索</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>您好，感谢您关注代理合作。了解到您所在地区是杭州，请问预计的合作规模如何？</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>高优先级；确认合作规模，准备代理政策和区域信息。</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>成功</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t>包含代理、合作或加盟关键词</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="M3" s="1" t="inlineStr"/>
+      <c r="N3" s="1" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
@@ -986,74 +1021,90 @@
   </sheetPr>
   <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>原始行号</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>导出用途</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>客户留言</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>联系方式</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>来源</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>意向等级</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>客户类型</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>线索阶段</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>客户回复</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>跟进动作</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>处理状态</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>判断依据</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>最终回复</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>回复状态</t>
         </is>
@@ -1072,86 +1123,90 @@
   </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>全部结果</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>包含原始数据和每行的 AI 处理结果；导出用途标记为草稿，仅供复核。</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>高意向</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>仅保留意向等级为“高”的客户，便于优先跟进。</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>处理状态非成功，或回复状态为“待复核”的行。</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>回复字段</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>客户回复是 AI 草稿；最终回复只有人工确认且通过导出安全检查后才可进入可发送文件；回复状态包括待确认、已确认、待复核。</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>线索阶段</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>线索阶段仅保存在当前浏览器会话，可选：新线索、已联系、待补信息、已转交；导出后由人工继续维护。</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>安全提示</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>请先脱敏并人工复核客户回复，再对外发送；原始行号用于追溯，不会导出 index、row_id 或 API key。</t>
         </is>

</xml_diff>